<commit_message>
Rond alle getallen af op 2 decimalen in output
</commit_message>
<xml_diff>
--- a/Aandelen Portfolio Rendement.xlsx
+++ b/Aandelen Portfolio Rendement.xlsx
@@ -473,25 +473,25 @@
         <v>71.5</v>
       </c>
       <c r="C2" t="n">
-        <v>9285.509999999998</v>
+        <v>9285.51</v>
       </c>
       <c r="D2" t="n">
-        <v>186.06</v>
+        <v>180.66</v>
       </c>
       <c r="E2" t="n">
-        <v>13303.29</v>
+        <v>12917.19</v>
       </c>
       <c r="F2" t="n">
         <v>129.8672727272727</v>
       </c>
       <c r="G2" t="n">
-        <v>4017.780000000002</v>
+        <v>3631.68</v>
       </c>
       <c r="H2" t="n">
-        <v>43.2693519257424</v>
+        <v>39.11</v>
       </c>
       <c r="I2" t="n">
-        <v>37.60090271855412</v>
+        <v>37.81</v>
       </c>
     </row>
     <row r="3">
@@ -507,22 +507,22 @@
         <v>3783.28</v>
       </c>
       <c r="D3" t="n">
-        <v>450.45</v>
+        <v>420.75</v>
       </c>
       <c r="E3" t="n">
-        <v>11441.43</v>
+        <v>10687.05</v>
       </c>
       <c r="F3" t="n">
         <v>148.948031496063</v>
       </c>
       <c r="G3" t="n">
-        <v>7658.149999999998</v>
+        <v>6903.77</v>
       </c>
       <c r="H3" t="n">
-        <v>202.4209151847074</v>
+        <v>182.48</v>
       </c>
       <c r="I3" t="n">
-        <v>32.33847389564135</v>
+        <v>31.29</v>
       </c>
     </row>
     <row r="4">
@@ -538,22 +538,22 @@
         <v>2016.03</v>
       </c>
       <c r="D4" t="n">
-        <v>355.55</v>
+        <v>343.7</v>
       </c>
       <c r="E4" t="n">
-        <v>2524.405</v>
+        <v>2440.27</v>
       </c>
       <c r="F4" t="n">
         <v>283.9478873239437</v>
       </c>
       <c r="G4" t="n">
-        <v>508.3749999999998</v>
+        <v>424.24</v>
       </c>
       <c r="H4" t="n">
-        <v>25.21663864129005</v>
+        <v>21.04</v>
       </c>
       <c r="I4" t="n">
-        <v>7.135070108764944</v>
+        <v>7.14</v>
       </c>
     </row>
     <row r="5">
@@ -569,22 +569,22 @@
         <v>3351.34</v>
       </c>
       <c r="D5" t="n">
-        <v>218.9</v>
+        <v>219.5</v>
       </c>
       <c r="E5" t="n">
-        <v>3874.53</v>
+        <v>3885.15</v>
       </c>
       <c r="F5" t="n">
         <v>189.3412429378531</v>
       </c>
       <c r="G5" t="n">
-        <v>523.1899999999996</v>
+        <v>533.8099999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>15.61136739334116</v>
+        <v>15.93</v>
       </c>
       <c r="I5" t="n">
-        <v>10.95111251503346</v>
+        <v>11.37</v>
       </c>
     </row>
     <row r="6">
@@ -603,19 +603,19 @@
         <v>14.548</v>
       </c>
       <c r="E6" t="n">
-        <v>2211.296</v>
+        <v>2211.3</v>
       </c>
       <c r="F6" t="n">
         <v>13.24671052631579</v>
       </c>
       <c r="G6" t="n">
-        <v>197.7959999999998</v>
+        <v>197.8</v>
       </c>
       <c r="H6" t="n">
-        <v>9.8234914328284</v>
+        <v>9.82</v>
       </c>
       <c r="I6" t="n">
-        <v>6.250087442875247</v>
+        <v>6.47</v>
       </c>
     </row>
     <row r="7">
@@ -631,22 +631,22 @@
         <v>1220.4</v>
       </c>
       <c r="D7" t="n">
-        <v>75.56999999999999</v>
+        <v>75.828</v>
       </c>
       <c r="E7" t="n">
-        <v>1284.69</v>
+        <v>1289.08</v>
       </c>
       <c r="F7" t="n">
         <v>71.78823529411764</v>
       </c>
       <c r="G7" t="n">
-        <v>64.28999999999996</v>
+        <v>68.68000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>5.267944936086526</v>
+        <v>5.63</v>
       </c>
       <c r="I7" t="n">
-        <v>3.631094542289861</v>
+        <v>3.77</v>
       </c>
     </row>
     <row r="8">
@@ -662,22 +662,22 @@
         <v>819.6</v>
       </c>
       <c r="D8" t="n">
-        <v>370.3</v>
+        <v>364.9</v>
       </c>
       <c r="E8" t="n">
-        <v>740.6</v>
+        <v>729.8</v>
       </c>
       <c r="F8" t="n">
         <v>409.8</v>
       </c>
       <c r="G8" t="n">
-        <v>-79</v>
+        <v>-89.8</v>
       </c>
       <c r="H8" t="n">
-        <v>-9.638848218643242</v>
+        <v>-10.96</v>
       </c>
       <c r="I8" t="n">
-        <v>2.093258776841006</v>
+        <v>2.14</v>
       </c>
     </row>
     <row r="9">
@@ -692,14 +692,14 @@
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>35380.241</v>
+        <v>34159.83</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
-        <v>12890.581</v>
+        <v>11670.17</v>
       </c>
       <c r="H9" t="n">
-        <v>57.31781182996986</v>
+        <v>51.89</v>
       </c>
       <c r="I9" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
Voeg snapshot_opslaan toe aan email_automatisering
</commit_message>
<xml_diff>
--- a/Aandelen Portfolio Rendement.xlsx
+++ b/Aandelen Portfolio Rendement.xlsx
@@ -476,22 +476,22 @@
         <v>9285.51</v>
       </c>
       <c r="D2" t="n">
-        <v>180.66</v>
+        <v>178.52</v>
       </c>
       <c r="E2" t="n">
-        <v>12917.19</v>
+        <v>12764.18</v>
       </c>
       <c r="F2" t="n">
         <v>129.8672727272727</v>
       </c>
       <c r="G2" t="n">
-        <v>3631.68</v>
+        <v>3478.67</v>
       </c>
       <c r="H2" t="n">
-        <v>39.11</v>
+        <v>37.46</v>
       </c>
       <c r="I2" t="n">
-        <v>37.81</v>
+        <v>37.4</v>
       </c>
     </row>
     <row r="3">
@@ -507,22 +507,22 @@
         <v>3783.28</v>
       </c>
       <c r="D3" t="n">
-        <v>420.75</v>
+        <v>444.35</v>
       </c>
       <c r="E3" t="n">
-        <v>10687.05</v>
+        <v>11286.49</v>
       </c>
       <c r="F3" t="n">
         <v>148.948031496063</v>
       </c>
       <c r="G3" t="n">
-        <v>6903.77</v>
+        <v>7503.21</v>
       </c>
       <c r="H3" t="n">
-        <v>182.48</v>
+        <v>198.33</v>
       </c>
       <c r="I3" t="n">
-        <v>31.29</v>
+        <v>33.07</v>
       </c>
     </row>
     <row r="4">
@@ -538,22 +538,22 @@
         <v>2016.03</v>
       </c>
       <c r="D4" t="n">
-        <v>343.7</v>
+        <v>330.4</v>
       </c>
       <c r="E4" t="n">
-        <v>2440.27</v>
+        <v>2345.84</v>
       </c>
       <c r="F4" t="n">
         <v>283.9478873239437</v>
       </c>
       <c r="G4" t="n">
-        <v>424.24</v>
+        <v>329.81</v>
       </c>
       <c r="H4" t="n">
-        <v>21.04</v>
+        <v>16.36</v>
       </c>
       <c r="I4" t="n">
-        <v>7.14</v>
+        <v>6.87</v>
       </c>
     </row>
     <row r="5">
@@ -569,22 +569,22 @@
         <v>3351.34</v>
       </c>
       <c r="D5" t="n">
-        <v>219.5</v>
+        <v>205.05</v>
       </c>
       <c r="E5" t="n">
-        <v>3885.15</v>
+        <v>3629.38</v>
       </c>
       <c r="F5" t="n">
         <v>189.3412429378531</v>
       </c>
       <c r="G5" t="n">
-        <v>533.8099999999999</v>
+        <v>278.05</v>
       </c>
       <c r="H5" t="n">
-        <v>15.93</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="I5" t="n">
-        <v>11.37</v>
+        <v>10.63</v>
       </c>
     </row>
     <row r="6">
@@ -600,22 +600,22 @@
         <v>2013.5</v>
       </c>
       <c r="D6" t="n">
-        <v>14.548</v>
+        <v>14.358</v>
       </c>
       <c r="E6" t="n">
-        <v>2211.3</v>
+        <v>2182.42</v>
       </c>
       <c r="F6" t="n">
         <v>13.24671052631579</v>
       </c>
       <c r="G6" t="n">
-        <v>197.8</v>
+        <v>168.92</v>
       </c>
       <c r="H6" t="n">
-        <v>9.82</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="I6" t="n">
-        <v>6.47</v>
+        <v>6.39</v>
       </c>
     </row>
     <row r="7">
@@ -631,22 +631,22 @@
         <v>1220.4</v>
       </c>
       <c r="D7" t="n">
-        <v>75.828</v>
+        <v>73.65000000000001</v>
       </c>
       <c r="E7" t="n">
-        <v>1289.08</v>
+        <v>1252.05</v>
       </c>
       <c r="F7" t="n">
         <v>71.78823529411764</v>
       </c>
       <c r="G7" t="n">
-        <v>68.68000000000001</v>
+        <v>31.65</v>
       </c>
       <c r="H7" t="n">
-        <v>5.63</v>
+        <v>2.59</v>
       </c>
       <c r="I7" t="n">
-        <v>3.77</v>
+        <v>3.67</v>
       </c>
     </row>
     <row r="8">
@@ -662,22 +662,22 @@
         <v>819.6</v>
       </c>
       <c r="D8" t="n">
-        <v>364.9</v>
+        <v>335.15</v>
       </c>
       <c r="E8" t="n">
-        <v>729.8</v>
+        <v>670.3</v>
       </c>
       <c r="F8" t="n">
         <v>409.8</v>
       </c>
       <c r="G8" t="n">
-        <v>-89.8</v>
+        <v>-149.3</v>
       </c>
       <c r="H8" t="n">
-        <v>-10.96</v>
+        <v>-18.22</v>
       </c>
       <c r="I8" t="n">
-        <v>2.14</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="9">
@@ -692,14 +692,14 @@
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>34159.83</v>
+        <v>34130.66</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
-        <v>11670.17</v>
+        <v>11641</v>
       </c>
       <c r="H9" t="n">
-        <v>51.89</v>
+        <v>51.76</v>
       </c>
       <c r="I9" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
Voeg mail_versturen toe aan email_automatisering en test succesvol
</commit_message>
<xml_diff>
--- a/Aandelen Portfolio Rendement.xlsx
+++ b/Aandelen Portfolio Rendement.xlsx
@@ -476,22 +476,22 @@
         <v>9285.51</v>
       </c>
       <c r="D2" t="n">
-        <v>178.52</v>
+        <v>181.84</v>
       </c>
       <c r="E2" t="n">
-        <v>12764.18</v>
+        <v>13001.56</v>
       </c>
       <c r="F2" t="n">
         <v>129.8672727272727</v>
       </c>
       <c r="G2" t="n">
-        <v>3478.67</v>
+        <v>3716.05</v>
       </c>
       <c r="H2" t="n">
-        <v>37.46</v>
+        <v>40.02</v>
       </c>
       <c r="I2" t="n">
-        <v>37.4</v>
+        <v>36.95</v>
       </c>
     </row>
     <row r="3">
@@ -507,22 +507,22 @@
         <v>3783.28</v>
       </c>
       <c r="D3" t="n">
-        <v>444.35</v>
+        <v>461.55</v>
       </c>
       <c r="E3" t="n">
-        <v>11286.49</v>
+        <v>11723.37</v>
       </c>
       <c r="F3" t="n">
         <v>148.948031496063</v>
       </c>
       <c r="G3" t="n">
-        <v>7503.21</v>
+        <v>7940.09</v>
       </c>
       <c r="H3" t="n">
-        <v>198.33</v>
+        <v>209.87</v>
       </c>
       <c r="I3" t="n">
-        <v>33.07</v>
+        <v>33.32</v>
       </c>
     </row>
     <row r="4">
@@ -538,22 +538,22 @@
         <v>2016.03</v>
       </c>
       <c r="D4" t="n">
-        <v>330.4</v>
+        <v>356.4</v>
       </c>
       <c r="E4" t="n">
-        <v>2345.84</v>
+        <v>2530.44</v>
       </c>
       <c r="F4" t="n">
         <v>283.9478873239437</v>
       </c>
       <c r="G4" t="n">
-        <v>329.81</v>
+        <v>514.41</v>
       </c>
       <c r="H4" t="n">
-        <v>16.36</v>
+        <v>25.52</v>
       </c>
       <c r="I4" t="n">
-        <v>6.87</v>
+        <v>7.19</v>
       </c>
     </row>
     <row r="5">
@@ -569,22 +569,22 @@
         <v>3351.34</v>
       </c>
       <c r="D5" t="n">
-        <v>205.05</v>
+        <v>210.7</v>
       </c>
       <c r="E5" t="n">
-        <v>3629.38</v>
+        <v>3729.39</v>
       </c>
       <c r="F5" t="n">
         <v>189.3412429378531</v>
       </c>
       <c r="G5" t="n">
-        <v>278.05</v>
+        <v>378.05</v>
       </c>
       <c r="H5" t="n">
-        <v>8.300000000000001</v>
+        <v>11.28</v>
       </c>
       <c r="I5" t="n">
-        <v>10.63</v>
+        <v>10.6</v>
       </c>
     </row>
     <row r="6">
@@ -600,22 +600,22 @@
         <v>2013.5</v>
       </c>
       <c r="D6" t="n">
-        <v>14.358</v>
+        <v>15.536</v>
       </c>
       <c r="E6" t="n">
-        <v>2182.42</v>
+        <v>2361.47</v>
       </c>
       <c r="F6" t="n">
         <v>13.24671052631579</v>
       </c>
       <c r="G6" t="n">
-        <v>168.92</v>
+        <v>347.97</v>
       </c>
       <c r="H6" t="n">
-        <v>8.390000000000001</v>
+        <v>17.28</v>
       </c>
       <c r="I6" t="n">
-        <v>6.39</v>
+        <v>6.71</v>
       </c>
     </row>
     <row r="7">
@@ -631,22 +631,22 @@
         <v>1220.4</v>
       </c>
       <c r="D7" t="n">
-        <v>73.65000000000001</v>
+        <v>69.68000000000001</v>
       </c>
       <c r="E7" t="n">
-        <v>1252.05</v>
+        <v>1184.56</v>
       </c>
       <c r="F7" t="n">
         <v>71.78823529411764</v>
       </c>
       <c r="G7" t="n">
-        <v>31.65</v>
+        <v>-35.84</v>
       </c>
       <c r="H7" t="n">
-        <v>2.59</v>
+        <v>-2.94</v>
       </c>
       <c r="I7" t="n">
-        <v>3.67</v>
+        <v>3.37</v>
       </c>
     </row>
     <row r="8">
@@ -662,22 +662,22 @@
         <v>819.6</v>
       </c>
       <c r="D8" t="n">
-        <v>335.15</v>
+        <v>327.2</v>
       </c>
       <c r="E8" t="n">
-        <v>670.3</v>
+        <v>654.4</v>
       </c>
       <c r="F8" t="n">
         <v>409.8</v>
       </c>
       <c r="G8" t="n">
-        <v>-149.3</v>
+        <v>-165.2</v>
       </c>
       <c r="H8" t="n">
-        <v>-18.22</v>
+        <v>-20.16</v>
       </c>
       <c r="I8" t="n">
-        <v>1.96</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="9">
@@ -692,14 +692,14 @@
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>34130.66</v>
+        <v>35185.19</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
-        <v>11641</v>
+        <v>12695.53</v>
       </c>
       <c r="H9" t="n">
-        <v>51.76</v>
+        <v>56.45</v>
       </c>
       <c r="I9" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
Voeg None-check toe aan vorige_snapshot_inlezen en claude_samenvatting_genereren
</commit_message>
<xml_diff>
--- a/Aandelen Portfolio Rendement.xlsx
+++ b/Aandelen Portfolio Rendement.xlsx
@@ -476,22 +476,22 @@
         <v>9285.51</v>
       </c>
       <c r="D2" t="n">
-        <v>181.84</v>
+        <v>181.82</v>
       </c>
       <c r="E2" t="n">
-        <v>13001.56</v>
+        <v>13000.13</v>
       </c>
       <c r="F2" t="n">
         <v>129.8672727272727</v>
       </c>
       <c r="G2" t="n">
-        <v>3716.05</v>
+        <v>3714.62</v>
       </c>
       <c r="H2" t="n">
-        <v>40.02</v>
+        <v>40</v>
       </c>
       <c r="I2" t="n">
-        <v>36.95</v>
+        <v>36.75</v>
       </c>
     </row>
     <row r="3">
@@ -507,22 +507,22 @@
         <v>3783.28</v>
       </c>
       <c r="D3" t="n">
-        <v>461.55</v>
+        <v>465.75</v>
       </c>
       <c r="E3" t="n">
-        <v>11723.37</v>
+        <v>11830.05</v>
       </c>
       <c r="F3" t="n">
         <v>148.948031496063</v>
       </c>
       <c r="G3" t="n">
-        <v>7940.09</v>
+        <v>8046.77</v>
       </c>
       <c r="H3" t="n">
-        <v>209.87</v>
+        <v>212.69</v>
       </c>
       <c r="I3" t="n">
-        <v>33.32</v>
+        <v>33.44</v>
       </c>
     </row>
     <row r="4">
@@ -538,19 +538,19 @@
         <v>2016.03</v>
       </c>
       <c r="D4" t="n">
-        <v>356.4</v>
+        <v>358.3</v>
       </c>
       <c r="E4" t="n">
-        <v>2530.44</v>
+        <v>2543.93</v>
       </c>
       <c r="F4" t="n">
         <v>283.9478873239437</v>
       </c>
       <c r="G4" t="n">
-        <v>514.41</v>
+        <v>527.9</v>
       </c>
       <c r="H4" t="n">
-        <v>25.52</v>
+        <v>26.19</v>
       </c>
       <c r="I4" t="n">
         <v>7.19</v>
@@ -569,22 +569,22 @@
         <v>3351.34</v>
       </c>
       <c r="D5" t="n">
-        <v>210.7</v>
+        <v>211.7</v>
       </c>
       <c r="E5" t="n">
-        <v>3729.39</v>
+        <v>3747.09</v>
       </c>
       <c r="F5" t="n">
         <v>189.3412429378531</v>
       </c>
       <c r="G5" t="n">
-        <v>378.05</v>
+        <v>395.75</v>
       </c>
       <c r="H5" t="n">
-        <v>11.28</v>
+        <v>11.81</v>
       </c>
       <c r="I5" t="n">
-        <v>10.6</v>
+        <v>10.59</v>
       </c>
     </row>
     <row r="6">
@@ -600,22 +600,22 @@
         <v>2013.5</v>
       </c>
       <c r="D6" t="n">
-        <v>15.536</v>
+        <v>15.842</v>
       </c>
       <c r="E6" t="n">
-        <v>2361.47</v>
+        <v>2407.98</v>
       </c>
       <c r="F6" t="n">
         <v>13.24671052631579</v>
       </c>
       <c r="G6" t="n">
-        <v>347.97</v>
+        <v>394.48</v>
       </c>
       <c r="H6" t="n">
-        <v>17.28</v>
+        <v>19.59</v>
       </c>
       <c r="I6" t="n">
-        <v>6.71</v>
+        <v>6.81</v>
       </c>
     </row>
     <row r="7">
@@ -646,7 +646,7 @@
         <v>-2.94</v>
       </c>
       <c r="I7" t="n">
-        <v>3.37</v>
+        <v>3.35</v>
       </c>
     </row>
     <row r="8">
@@ -662,22 +662,22 @@
         <v>819.6</v>
       </c>
       <c r="D8" t="n">
-        <v>327.2</v>
+        <v>330.1</v>
       </c>
       <c r="E8" t="n">
-        <v>654.4</v>
+        <v>660.2</v>
       </c>
       <c r="F8" t="n">
         <v>409.8</v>
       </c>
       <c r="G8" t="n">
-        <v>-165.2</v>
+        <v>-159.4</v>
       </c>
       <c r="H8" t="n">
-        <v>-20.16</v>
+        <v>-19.45</v>
       </c>
       <c r="I8" t="n">
-        <v>1.86</v>
+        <v>1.87</v>
       </c>
     </row>
     <row r="9">
@@ -692,14 +692,14 @@
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>35185.19</v>
+        <v>35373.94</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
-        <v>12695.53</v>
+        <v>12884.28</v>
       </c>
       <c r="H9" t="n">
-        <v>56.45</v>
+        <v>57.29</v>
       </c>
       <c r="I9" t="n">
         <v>100</v>

</xml_diff>